<commit_message>
Process in one step - local optimisation
</commit_message>
<xml_diff>
--- a/tests/simple_example/problem_definition.xlsx
+++ b/tests/simple_example/problem_definition.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="19029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Work\OneDrive - Transport Systems Catapult\Research\PhD\Models\tripchains_from_ODs\tests\simple_example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="DAD190B78EB412C7C7198C30A7DC985DF17920D9" xr6:coauthVersionLast="28" xr6:coauthVersionMax="28" xr10:uidLastSave="{831E1ADA-281E-463E-8935-723513455BFF}"/>
+  <xr:revisionPtr revIDLastSave="101" documentId="DAD190B78EB412C7C7198C30A7DC985DF17920D9" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{6737EC9D-0CA0-4D14-AC0F-80557975CD9F}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210" xr2:uid="{F6A259FC-2D38-4842-AE1E-E2802FA79334}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="179017"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="17">
   <si>
     <t>HA</t>
   </si>
@@ -67,6 +67,15 @@
   </si>
   <si>
     <t>b</t>
+  </si>
+  <si>
+    <t>Times</t>
+  </si>
+  <si>
+    <t>ResultTrips</t>
+  </si>
+  <si>
+    <t>ResultTimes</t>
   </si>
 </sst>
 </file>
@@ -109,7 +118,13 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="5">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -133,13 +148,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1D70010B-F1B6-4368-8732-96EB6CD062A0}" name="chains_formation" displayName="chains_formation" ref="B2:D16" totalsRowShown="0">
-  <autoFilter ref="B2:D16" xr:uid="{C0837855-CD0B-4A99-A767-2670B631291D}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1D70010B-F1B6-4368-8732-96EB6CD062A0}" name="chains_formation" displayName="chains_formation" ref="B2:E16" totalsRowShown="0">
+  <autoFilter ref="B2:E16" xr:uid="{C0837855-CD0B-4A99-A767-2670B631291D}"/>
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{B717F6FC-CFC4-4E1F-A08C-D62C81B6FEA8}" name="ChainID"/>
     <tableColumn id="2" xr3:uid="{4046632C-2D3E-4188-8212-4C0473070B04}" name="LegID"/>
-    <tableColumn id="3" xr3:uid="{C2511672-113D-4F46-A693-4A8D9E7DBC9D}" name="Trips" dataDxfId="2">
-      <calculatedColumnFormula>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{C2511672-113D-4F46-A693-4A8D9E7DBC9D}" name="Trips" dataDxfId="4">
+      <calculatedColumnFormula>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{6EB1A1D1-16AF-4E31-B4A3-0CFA6C42D61A}" name="ResultTrips" dataDxfId="3">
+      <calculatedColumnFormula>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -147,24 +165,28 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{88AAEA1A-2DDC-474B-A9A4-CFDBC1382CF2}" name="chain_trips" displayName="chain_trips" ref="F2:H7" totalsRowShown="0">
-  <autoFilter ref="F2:H7" xr:uid="{6ADC1CE1-B464-495C-9388-A48AF1658B2B}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{88AAEA1A-2DDC-474B-A9A4-CFDBC1382CF2}" name="chain_trips" displayName="chain_trips" ref="G2:J7" totalsRowShown="0">
+  <autoFilter ref="G2:J7" xr:uid="{6ADC1CE1-B464-495C-9388-A48AF1658B2B}"/>
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{CBC57893-FF1C-47ED-AE3C-15E113A53227}" name="ChainID"/>
     <tableColumn id="3" xr3:uid="{DDF6138B-39BB-4E75-894E-233EC5A99FDE}" name="Group"/>
-    <tableColumn id="2" xr3:uid="{ED9AD6EC-FBF8-45C7-BC92-DB5B3624FFE4}" name="Trips"/>
+    <tableColumn id="2" xr3:uid="{ED9AD6EC-FBF8-45C7-BC92-DB5B3624FFE4}" name="Times"/>
+    <tableColumn id="5" xr3:uid="{79F67609-B3EE-45AD-B03E-021A8537CA9F}" name="ResultTimes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D4C8C218-BDE3-46AD-ACB9-D3D277FA6537}" name="Table4" displayName="Table4" ref="J2:K10" totalsRowCount="1">
-  <autoFilter ref="J2:K9" xr:uid="{781A71C3-0098-4A62-87FD-B971F89B3F29}"/>
-  <tableColumns count="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D4C8C218-BDE3-46AD-ACB9-D3D277FA6537}" name="Table4" displayName="Table4" ref="L2:N10" totalsRowCount="1">
+  <autoFilter ref="L2:N9" xr:uid="{781A71C3-0098-4A62-87FD-B971F89B3F29}"/>
+  <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{50CE5110-E79E-4474-B33B-C271B8F81E94}" name="OD_pair"/>
-    <tableColumn id="2" xr3:uid="{A78BF333-93E7-4BFC-9973-105174CEDC06}" name="Trips" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0">
+    <tableColumn id="2" xr3:uid="{A78BF333-93E7-4BFC-9973-105174CEDC06}" name="Trips" totalsRowFunction="sum" dataDxfId="2" totalsRowDxfId="1">
       <calculatedColumnFormula>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[Trips])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{8D3D076F-3D4F-4783-8CDA-5711EF8693F4}" name="ResultTrips" totalsRowFunction="sum" dataDxfId="0">
+      <calculatedColumnFormula>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[ResultTrips])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -468,17 +490,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E865A3A8-F0B5-4FCE-819D-BAFDF87706B7}">
-  <dimension ref="B2:K16"/>
+  <dimension ref="B2:N16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="5" max="5" width="6.140625" customWidth="1"/>
-    <col min="6" max="7" width="10" customWidth="1"/>
-    <col min="9" max="9" width="7" customWidth="1"/>
-    <col min="10" max="10" width="10.28515625" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.140625" customWidth="1"/>
+    <col min="7" max="8" width="10" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7" customWidth="1"/>
+    <col min="12" max="12" width="10.28515625" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>6</v>
       </c>
@@ -488,23 +514,32 @@
       <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" t="s">
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s">
         <v>6</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>11</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" t="s">
+        <v>16</v>
+      </c>
+      <c r="L2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" t="s">
         <v>7</v>
       </c>
-      <c r="J2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="N2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>1</v>
       </c>
@@ -512,27 +547,38 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</f>
-        <v>5</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3" t="s">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</f>
+        <v>5</v>
+      </c>
+      <c r="E3">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</f>
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
         <v>12</v>
       </c>
-      <c r="H3">
-        <v>5</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="I3">
+        <v>5</v>
+      </c>
+      <c r="J3">
+        <v>4</v>
+      </c>
+      <c r="L3" t="s">
         <v>0</v>
       </c>
-      <c r="K3">
+      <c r="M3">
         <f>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[Trips])</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="N3">
+        <f>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[ResultTrips])</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>1</v>
       </c>
@@ -540,27 +586,38 @@
         <v>1</v>
       </c>
       <c r="D4">
-        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</f>
-        <v>5</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-      <c r="G4" t="s">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</f>
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</f>
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4" t="s">
         <v>12</v>
       </c>
-      <c r="H4">
-        <v>2</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="I4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="L4" t="s">
         <v>10</v>
       </c>
-      <c r="K4">
+      <c r="M4">
         <f>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[Trips])</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="N4">
+        <f>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[ResultTrips])</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B5">
         <v>1</v>
       </c>
@@ -568,27 +625,38 @@
         <v>5</v>
       </c>
       <c r="D5">
-        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</f>
-        <v>5</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-      <c r="G5" t="s">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</f>
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</f>
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
+      </c>
+      <c r="H5" t="s">
         <v>13</v>
       </c>
-      <c r="H5">
-        <v>3</v>
-      </c>
-      <c r="J5" t="s">
-        <v>1</v>
-      </c>
-      <c r="K5">
+      <c r="I5">
+        <v>3</v>
+      </c>
+      <c r="J5">
+        <v>4</v>
+      </c>
+      <c r="L5" t="s">
+        <v>1</v>
+      </c>
+      <c r="M5">
         <f>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[Trips])</f>
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="N5">
+        <f>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[ResultTrips])</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>2</v>
       </c>
@@ -596,27 +664,38 @@
         <v>0</v>
       </c>
       <c r="D6">
-        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</f>
-        <v>2</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="G6" t="s">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</f>
+        <v>2</v>
+      </c>
+      <c r="E6">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</f>
+        <v>2</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6" t="s">
         <v>13</v>
       </c>
-      <c r="H6">
-        <v>4</v>
-      </c>
-      <c r="J6" t="s">
-        <v>2</v>
-      </c>
-      <c r="K6">
+      <c r="I6">
+        <v>4</v>
+      </c>
+      <c r="J6">
+        <v>5</v>
+      </c>
+      <c r="L6" t="s">
+        <v>2</v>
+      </c>
+      <c r="M6">
         <f>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[Trips])</f>
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="N6">
+        <f>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[ResultTrips])</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>2</v>
       </c>
@@ -624,27 +703,35 @@
         <v>10</v>
       </c>
       <c r="D7">
-        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</f>
-        <v>2</v>
-      </c>
-      <c r="F7">
-        <v>5</v>
-      </c>
-      <c r="G7" t="s">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</f>
+        <v>2</v>
+      </c>
+      <c r="E7">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</f>
+        <v>2</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="H7" t="s">
         <v>13</v>
       </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="J7" t="s">
-        <v>3</v>
-      </c>
-      <c r="K7">
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="L7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M7">
         <f>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[Trips])</f>
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="N7">
+        <f>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[ResultTrips])</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>3</v>
       </c>
@@ -652,18 +739,26 @@
         <v>0</v>
       </c>
       <c r="D8">
-        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</f>
-        <v>3</v>
-      </c>
-      <c r="J8" t="s">
-        <v>4</v>
-      </c>
-      <c r="K8">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</f>
+        <v>3</v>
+      </c>
+      <c r="E8">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</f>
+        <v>4</v>
+      </c>
+      <c r="L8" t="s">
+        <v>4</v>
+      </c>
+      <c r="M8">
         <f>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[Trips])</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="N8">
+        <f>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[ResultTrips])</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>3</v>
       </c>
@@ -671,18 +766,26 @@
         <v>1</v>
       </c>
       <c r="D9">
-        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</f>
-        <v>3</v>
-      </c>
-      <c r="J9" t="s">
-        <v>5</v>
-      </c>
-      <c r="K9">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</f>
+        <v>3</v>
+      </c>
+      <c r="E9">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</f>
+        <v>4</v>
+      </c>
+      <c r="L9" t="s">
+        <v>5</v>
+      </c>
+      <c r="M9">
         <f>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[Trips])</f>
         <v>9</v>
       </c>
-    </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="N9">
+        <f>SUMIF(chains_formation[LegID],Table4[[#This Row],[OD_pair]],chains_formation[ResultTrips])</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>3</v>
       </c>
@@ -690,15 +793,23 @@
         <v>2</v>
       </c>
       <c r="D10">
-        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</f>
-        <v>3</v>
-      </c>
-      <c r="K10" s="1">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</f>
+        <v>3</v>
+      </c>
+      <c r="E10">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</f>
+        <v>4</v>
+      </c>
+      <c r="M10" s="1">
         <f>SUBTOTAL(109,Table4[Trips])</f>
         <v>42</v>
       </c>
-    </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="N10">
+        <f>SUBTOTAL(109,Table4[ResultTrips])</f>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>3</v>
       </c>
@@ -706,11 +817,15 @@
         <v>3</v>
       </c>
       <c r="D11">
-        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</f>
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>4</v>
       </c>
@@ -718,11 +833,15 @@
         <v>4</v>
       </c>
       <c r="D12">
-        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</f>
+        <v>4</v>
+      </c>
+      <c r="E12">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>4</v>
       </c>
@@ -730,11 +849,15 @@
         <v>5</v>
       </c>
       <c r="D13">
-        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</f>
+        <v>4</v>
+      </c>
+      <c r="E13">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B14">
         <v>5</v>
       </c>
@@ -742,11 +865,15 @@
         <v>4</v>
       </c>
       <c r="D14">
-        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</f>
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B15">
         <v>5</v>
       </c>
@@ -754,11 +881,15 @@
         <v>2</v>
       </c>
       <c r="D15">
-        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</f>
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B16">
         <v>5</v>
       </c>
@@ -766,8 +897,12 @@
         <v>3</v>
       </c>
       <c r="D16">
-        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Trips])</f>
-        <v>1</v>
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[Times])</f>
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <f>SUMIF(chain_trips[ChainID],chains_formation[ChainID],chain_trips[ResultTimes])</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>